<commit_message>
feat: fix apriltag resolution
</commit_message>
<xml_diff>
--- a/fiducial_markers/apriltag/data/apriltag_resolution_chart.xlsx
+++ b/fiducial_markers/apriltag/data/apriltag_resolution_chart.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danielwliu/Dev/Python/Projects/Learning/pearl-lab-software-dev/fiducial_markers/apriltag/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDDF0DE4-1402-954F-A0FC-660A73EE1BDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F7AC9D8-1BFC-364F-8052-48F33B65784E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3440" yWindow="1540" windowWidth="30240" windowHeight="17520" xr2:uid="{ABFF90C4-89F4-FE48-B797-A3B896040CD6}"/>
+    <workbookView xWindow="0" yWindow="4160" windowWidth="30240" windowHeight="17520" xr2:uid="{ABFF90C4-89F4-FE48-B797-A3B896040CD6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="8">
   <si>
     <t>Resolution (px)</t>
   </si>
@@ -44,18 +44,9 @@
     <t>1280 x 720</t>
   </si>
   <si>
-    <t>1536 x 864</t>
-  </si>
-  <si>
     <t>Average Detection Confidence</t>
   </si>
   <si>
-    <t>1366 x 768</t>
-  </si>
-  <si>
-    <t>1600 x 900</t>
-  </si>
-  <si>
     <t>1440 x 900</t>
   </si>
   <si>
@@ -65,13 +56,10 @@
     <t>Average Accuracy (%)</t>
   </si>
   <si>
-    <t>720 x 480</t>
-  </si>
-  <si>
     <t>640 x 480 (SD)</t>
   </si>
   <si>
-    <t>1920 x 1080 (FULL HD)</t>
+    <t>1920 1080</t>
   </si>
 </sst>
 </file>
@@ -451,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E3D848C-7F5F-0C45-B111-88E0E7DADCD2}">
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="8" width="25.83203125" customWidth="1"/>
@@ -462,36 +450,36 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E1" t="s">
         <v>0</v>
       </c>
       <c r="F1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B2">
         <v>25</v>
       </c>
       <c r="E2" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F2">
         <v>25</v>
@@ -553,76 +541,6 @@
         <v>200</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10">
-        <v>25</v>
-      </c>
-      <c r="E10" t="s">
-        <v>2</v>
-      </c>
-      <c r="F10">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B11">
-        <v>50</v>
-      </c>
-      <c r="F11">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B12">
-        <v>75</v>
-      </c>
-      <c r="F12">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B13">
-        <v>100</v>
-      </c>
-      <c r="F13">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B14">
-        <v>125</v>
-      </c>
-      <c r="F14">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B15">
-        <v>150</v>
-      </c>
-      <c r="F15">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="B16">
-        <v>175</v>
-      </c>
-      <c r="F16">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B17">
-        <v>200</v>
-      </c>
-      <c r="F17">
-        <v>200</v>
-      </c>
-    </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>1</v>
@@ -631,7 +549,7 @@
         <v>25</v>
       </c>
       <c r="E18" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F18">
         <v>25</v>
@@ -690,76 +608,6 @@
         <v>200</v>
       </c>
       <c r="F25">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
-        <v>4</v>
-      </c>
-      <c r="B26">
-        <v>25</v>
-      </c>
-      <c r="E26" t="s">
-        <v>11</v>
-      </c>
-      <c r="F26">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B27">
-        <v>50</v>
-      </c>
-      <c r="F27">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B28">
-        <v>75</v>
-      </c>
-      <c r="F28">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B29">
-        <v>100</v>
-      </c>
-      <c r="F29">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B30">
-        <v>125</v>
-      </c>
-      <c r="F30">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B31">
-        <v>150</v>
-      </c>
-      <c r="F31">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B32">
-        <v>175</v>
-      </c>
-      <c r="F32">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B33">
-        <v>200</v>
-      </c>
-      <c r="F33">
         <v>200</v>
       </c>
     </row>

</xml_diff>